<commit_message>
disable table filter button and adjust formatting
</commit_message>
<xml_diff>
--- a/shrinking-dropdown/shrinking-dropdown.xlsx
+++ b/shrinking-dropdown/shrinking-dropdown.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/amin/Personal/excel repo files/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/amin/Personal/github/excel-solutions/shrinking-dropdown/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96403F38-0A2B-FF4C-B84C-80B05D28F37A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEBD017E-B14C-F947-A350-41E6A9AE4AE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="20400" xr2:uid="{CDC59B7F-BA3E-1E4B-A0A6-6340F8BA902D}"/>
   </bookViews>
@@ -264,20 +264,42 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="centerContinuous" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="10">
+    <dxf>
+      <font>
+        <b/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="6" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <font>
         <strike val="0"/>
@@ -370,21 +392,6 @@
       </font>
     </dxf>
     <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <border>
         <vertical/>
       </border>
@@ -413,7 +420,7 @@
     </dxf>
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
-    <tableStyle name="TableStyleLight11 less border" pivot="0" count="5" xr9:uid="{88147DB1-91F6-E84A-A54E-D5B7DE2E4346}">
+    <tableStyle name="TableStyleLight11 less border" pivot="0" count="3" xr9:uid="{88147DB1-91F6-E84A-A54E-D5B7DE2E4346}">
       <tableStyleElement type="wholeTable" dxfId="9"/>
       <tableStyleElement type="firstRowStripe" dxfId="8"/>
       <tableStyleElement type="secondRowStripe" dxfId="7"/>
@@ -790,21 +797,24 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{AE4692D7-91FD-E44A-8D0D-1595BC75CCBB}" name="PersonTaskTbl" displayName="PersonTaskTbl" ref="F2:G16" totalsRowShown="0" headerRowDxfId="6" dataDxfId="5">
-  <autoFilter ref="F2:G16" xr:uid="{AE4692D7-91FD-E44A-8D0D-1595BC75CCBB}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{AE4692D7-91FD-E44A-8D0D-1595BC75CCBB}" name="PersonTaskTbl" displayName="PersonTaskTbl" ref="F2:G16" totalsRowShown="0" headerRowDxfId="0" dataDxfId="6">
+  <autoFilter ref="F2:G16" xr:uid="{AE4692D7-91FD-E44A-8D0D-1595BC75CCBB}">
+    <filterColumn colId="0" hiddenButton="1"/>
+    <filterColumn colId="1" hiddenButton="1"/>
+  </autoFilter>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{0A131958-061B-F84B-8488-EA81BF6CA636}" name="Person Name" dataDxfId="4"/>
-    <tableColumn id="2" xr3:uid="{0A7CC692-FB35-6245-8FCA-713D6F1C408A}" name="Assigned Task" dataDxfId="3"/>
+    <tableColumn id="1" xr3:uid="{0A131958-061B-F84B-8488-EA81BF6CA636}" name="Person Name" dataDxfId="5"/>
+    <tableColumn id="2" xr3:uid="{0A7CC692-FB35-6245-8FCA-713D6F1C408A}" name="Assigned Task" dataDxfId="4"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight11 less border" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{1760D98C-7D9B-E44A-8FD0-B66DD9E4AFA9}" name="TaskTbl" displayName="TaskTbl" ref="B2:B16" totalsRowShown="0" headerRowDxfId="2" dataDxfId="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{1760D98C-7D9B-E44A-8FD0-B66DD9E4AFA9}" name="TaskTbl" displayName="TaskTbl" ref="B2:B16" totalsRowShown="0" headerRowDxfId="3" dataDxfId="2">
   <autoFilter ref="B2:B16" xr:uid="{1760D98C-7D9B-E44A-8FD0-B66DD9E4AFA9}"/>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{DBB0F81E-C311-924C-8E0C-6420004AAFD9}" name="Task Name" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{DBB0F81E-C311-924C-8E0C-6420004AAFD9}" name="Task Name" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1140,10 +1150,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" s="1" customFormat="1" ht="34" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F1" s="9" t="s">
+      <c r="F1" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="G1" s="9"/>
+      <c r="G1" s="8"/>
     </row>
     <row r="2" spans="1:7" ht="25" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2"/>
@@ -1151,14 +1161,14 @@
         <v>26</v>
       </c>
       <c r="C2" s="2"/>
-      <c r="D2" s="8" t="s">
+      <c r="D2" s="7" t="s">
         <v>27</v>
       </c>
       <c r="E2" s="1"/>
-      <c r="F2" s="7" t="s">
+      <c r="F2" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="7" t="s">
+      <c r="G2" s="9" t="s">
         <v>25</v>
       </c>
     </row>

</xml_diff>